<commit_message>
modify lat and lon for one property
</commit_message>
<xml_diff>
--- a/properties.xlsx
+++ b/properties.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Jobs\Las Brisas PM\las-brisas-mapa\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDC7A082-4785-41D1-AE02-D5C572C8C323}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D25DF79F-626A-4C71-8AB8-4FE8EE8BECD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,20 @@
     <sheet name="properties" sheetId="1" r:id="rId1"/>
     <sheet name="property_lot" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -976,10 +989,10 @@
         <v>23</v>
       </c>
       <c r="G9" s="2">
-        <v>18.410553752416501</v>
+        <v>18.4105130335677</v>
       </c>
       <c r="H9" s="2">
-        <v>-66.057143028835199</v>
+        <v>-66.057084020239998</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>66</v>

</xml_diff>